<commit_message>
feat(publication): update generate_table6.py to compute metrics dynamically from raw data with micro-average aggregation
</commit_message>
<xml_diff>
--- a/publication/results/tables/table6_random_seed_invariance.xlsx
+++ b/publication/results/tables/table6_random_seed_invariance.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,12 +418,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metadata Field</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -509,7 +497,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>publication/scripts/generate_table6.py</t>
+          <t>publication/scripts/generate_table6.py (Computed dynamically from raw.xlsx)</t>
         </is>
       </c>
     </row>
@@ -528,22 +516,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset &amp; Evaluation Protocol</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Random Seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Primary Tier: Strict Exact F1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Secondary Tier: Adapted ADE F1</t>
         </is>
@@ -562,12 +550,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.5582 ± 0.0649</t>
+          <t>0.5470</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.7431 ± 0.0295</t>
+          <t>0.7402</t>
         </is>
       </c>
     </row>
@@ -584,12 +572,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.5652 ± 0.0509</t>
+          <t>0.5524</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.7402 ± 0.0293</t>
+          <t>0.7369</t>
         </is>
       </c>
     </row>
@@ -606,12 +594,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.5783 ± 0.0697</t>
+          <t>0.5636</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.7586 ± 0.0355</t>
+          <t>0.7523</t>
         </is>
       </c>
     </row>
@@ -628,12 +616,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.5663 ± 0.0476</t>
+          <t>0.5571</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.7413 ± 0.0324</t>
+          <t>0.7386</t>
         </is>
       </c>
     </row>
@@ -650,12 +638,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.5748 ± 0.0694</t>
+          <t>0.5620</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.7484 ± 0.0371</t>
+          <t>0.7422</t>
         </is>
       </c>
     </row>
@@ -672,12 +660,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.5685 ± 0.0080</t>
+          <t>0.5564 ± 0.0069</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.7463 ± 0.0075</t>
+          <t>0.7420 ± 0.0061</t>
         </is>
       </c>
     </row>

</xml_diff>